<commit_message>
Document PubMachineCountyCase in English and refresh case crop labels.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data-raw/data-tidy/public-site/moa-machine-county/xlsx/case-year-2022-batch02.xlsx
+++ b/data-raw/data-tidy/public-site/moa-machine-county/xlsx/case-year-2022-batch02.xlsx
@@ -119,7 +119,7 @@
     <t xml:space="preserve">南丰</t>
   </si>
   <si>
-    <t xml:space="preserve">金秋砂糖桔</t>
+    <t xml:space="preserve">砂糖桔</t>
   </si>
   <si>
     <t xml:space="preserve">湖北宜昌柑橘机械化生产模式与典型案例</t>
@@ -197,7 +197,7 @@
     <t xml:space="preserve">贺兰山东麓</t>
   </si>
   <si>
-    <t xml:space="preserve">酿酒葡萄</t>
+    <t xml:space="preserve">葡萄</t>
   </si>
   <si>
     <t xml:space="preserve">新疆玛纳斯酿酒葡萄机械化生产模式与典型案例</t>
@@ -239,7 +239,7 @@
     <t xml:space="preserve">安吉</t>
   </si>
   <si>
-    <t xml:space="preserve">白化茶</t>
+    <t xml:space="preserve">白茶</t>
   </si>
   <si>
     <t xml:space="preserve">浙北缓坡白化茶（安吉雅思清和）机械化生产模式与典型案例</t>

</xml_diff>